<commit_message>
Redo Vercelli Tav. 10: real double reading, 0 validation flags
Re-run with 01b (Senza/TOTALE block location), pass 1 from OCR (01c),
independent visual pass 2 of the strip crops, disagreements decided by
check_pass.py (both block sum and Tav. 1 sum) or by zoomed re-read.
flags_vercelli.csv is empty; tav10_vercelli.dta rebuilt from the validated data.
See docs/audit_2026-10.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011mvLWFfLFbnKm7v6S9L2EZ
</commit_message>
<xml_diff>
--- a/output/tav10_vercelli.xlsx
+++ b/output/tav10_vercelli.xlsx
@@ -855,7 +855,7 @@
         <v>83.48999999999999</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="S2" t="n">
         <v>98.37</v>
@@ -960,7 +960,7 @@
         <v>40</v>
       </c>
       <c r="BA2" t="n">
-        <v>771.4400000000001</v>
+        <v>1771.44</v>
       </c>
       <c r="BB2" t="n">
         <v>65</v>
@@ -969,46 +969,46 @@
         <v>4066.16</v>
       </c>
       <c r="BD2" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BE2" t="n">
-        <v>0</v>
+        <v>2638.21</v>
       </c>
       <c r="BF2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="BG2" t="n">
-        <v>0</v>
+        <v>2056.49</v>
       </c>
       <c r="BH2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BI2" t="n">
-        <v>0</v>
+        <v>890.15</v>
       </c>
       <c r="BJ2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>444.27</v>
+      </c>
+      <c r="BL2" t="n">
         <v>9</v>
       </c>
-      <c r="BK2" t="n">
+      <c r="BM2" t="n">
         <v>3363.38</v>
       </c>
-      <c r="BL2" t="n">
+      <c r="BN2" t="n">
         <v>8</v>
       </c>
-      <c r="BM2" t="n">
+      <c r="BO2" t="n">
         <v>5627.36</v>
       </c>
-      <c r="BN2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO2" t="n">
+      <c r="BP2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ2" t="n">
         <v>1262.59</v>
-      </c>
-      <c r="BP2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ2" t="n">
-        <v>0</v>
       </c>
       <c r="BR2" t="n">
         <v>0</v>
@@ -1151,7 +1151,9 @@
       <c r="AJ3" t="n">
         <v>420</v>
       </c>
-      <c r="AK3" t="inlineStr"/>
+      <c r="AK3" t="n">
+        <v>2551.35</v>
+      </c>
       <c r="AL3" t="n">
         <v>214</v>
       </c>
@@ -1165,7 +1167,7 @@
         <v>1219.63</v>
       </c>
       <c r="AP3" t="n">
-        <v>5</v>
+        <v>59</v>
       </c>
       <c r="AQ3" t="n">
         <v>800.99</v>
@@ -1195,58 +1197,58 @@
         <v>611.64</v>
       </c>
       <c r="AZ3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="BA3" t="n">
         <v>685.3200000000001</v>
       </c>
       <c r="BB3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="BC3" t="n">
-        <v>0</v>
+        <v>548.63</v>
       </c>
       <c r="BD3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="BE3" t="n">
-        <v>0</v>
+        <v>629.17</v>
       </c>
       <c r="BF3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="BG3" t="n">
-        <v>0</v>
+        <v>1032.59</v>
       </c>
       <c r="BH3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BI3" t="n">
+        <v>501.24</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK3" t="n">
         <v>213.28</v>
       </c>
-      <c r="BJ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK3" t="n">
+      <c r="BL3" t="n">
+        <v>5</v>
+      </c>
+      <c r="BM3" t="n">
         <v>1970.93</v>
       </c>
-      <c r="BL3" t="n">
+      <c r="BN3" t="n">
         <v>6</v>
       </c>
-      <c r="BM3" t="n">
+      <c r="BO3" t="n">
         <v>4238.49</v>
       </c>
-      <c r="BN3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO3" t="n">
+      <c r="BP3" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ3" t="n">
         <v>4383.08</v>
-      </c>
-      <c r="BP3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ3" t="n">
-        <v>0</v>
       </c>
       <c r="BR3" t="n">
         <v>0</v>
@@ -1291,7 +1293,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -1405,88 +1407,88 @@
         <v>190</v>
       </c>
       <c r="AP4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0</v>
+        <v>121.92</v>
       </c>
       <c r="AR4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="AS4" t="n">
-        <v>0</v>
+        <v>206.71</v>
       </c>
       <c r="AT4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU4" t="n">
+        <v>134.62</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW4" t="n">
         <v>77.70999999999999</v>
       </c>
-      <c r="AV4" t="n">
+      <c r="AX4" t="n">
         <v>4</v>
       </c>
-      <c r="AW4" t="n">
+      <c r="AY4" t="n">
         <v>138.14</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="AZ4" t="n">
         <v>3</v>
       </c>
-      <c r="AY4" t="n">
+      <c r="BA4" t="n">
         <v>133.51</v>
       </c>
-      <c r="AZ4" t="n">
+      <c r="BB4" t="n">
         <v>6</v>
       </c>
-      <c r="BA4" t="n">
+      <c r="BC4" t="n">
         <v>404.23</v>
       </c>
-      <c r="BB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC4" t="n">
+      <c r="BD4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BE4" t="n">
         <v>431.45</v>
-      </c>
-      <c r="BD4" t="n">
-        <v>2</v>
-      </c>
-      <c r="BE4" t="n">
-        <v>234.85</v>
       </c>
       <c r="BF4" t="n">
         <v>2</v>
       </c>
       <c r="BG4" t="n">
+        <v>234.85</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI4" t="n">
         <v>377.56</v>
       </c>
-      <c r="BH4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI4" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL4" t="n">
         <v>7</v>
       </c>
-      <c r="BK4" t="n">
+      <c r="BM4" t="n">
         <v>2553.78</v>
       </c>
-      <c r="BL4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM4" t="n">
+      <c r="BN4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO4" t="n">
         <v>691.1799999999999</v>
       </c>
-      <c r="BN4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO4" t="n">
+      <c r="BP4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ4" t="n">
         <v>1096</v>
-      </c>
-      <c r="BP4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ4" t="n">
-        <v>0</v>
       </c>
       <c r="BR4" t="n">
         <v>0</v>
@@ -1497,7 +1499,9 @@
       <c r="BT4" t="n">
         <v>4881</v>
       </c>
-      <c r="BU4" t="inlineStr"/>
+      <c r="BU4" t="n">
+        <v>12136.05</v>
+      </c>
       <c r="BV4" t="inlineStr">
         <is>
           <t>M</t>
@@ -1549,7 +1553,9 @@
       <c r="J5" t="n">
         <v>108</v>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>27.5</v>
+      </c>
       <c r="L5" t="n">
         <v>76</v>
       </c>
@@ -1689,19 +1695,19 @@
         <v>0</v>
       </c>
       <c r="BF5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG5" t="n">
         <v>146.21</v>
       </c>
       <c r="BH5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BI5" t="n">
         <v>167.47</v>
       </c>
       <c r="BJ5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BK5" t="n">
         <v>229</v>
@@ -1731,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="BT5" t="n">
-        <v>0</v>
+        <v>1569</v>
       </c>
       <c r="BU5" t="n">
-        <v>0</v>
+        <v>7018.63</v>
       </c>
       <c r="BV5" t="inlineStr">
         <is>
@@ -1775,20 +1781,26 @@
       <c r="F6" t="n">
         <v>1369</v>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>90.06</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1204</v>
+      </c>
       <c r="I6" t="n">
         <v>186.13</v>
       </c>
       <c r="J6" t="n">
         <v>963</v>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>245.58</v>
+      </c>
       <c r="L6" t="n">
         <v>798</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>285.09</v>
       </c>
       <c r="N6" t="n">
         <v>635</v>
@@ -1800,151 +1812,163 @@
         <v>1282</v>
       </c>
       <c r="Q6" t="n">
+        <v>797.77</v>
+      </c>
+      <c r="R6" t="n">
+        <v>1077</v>
+      </c>
+      <c r="S6" t="n">
         <v>943.09</v>
       </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
       <c r="T6" t="n">
-        <v>0</v>
+        <v>1426</v>
       </c>
       <c r="U6" t="n">
-        <v>0</v>
+        <v>1772.95</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>1926.25</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>873</v>
       </c>
       <c r="Y6" t="n">
-        <v>1814.86</v>
+        <v>1969.36</v>
       </c>
       <c r="Z6" t="n">
-        <v>0</v>
+        <v>682</v>
       </c>
       <c r="AA6" t="n">
+        <v>1874.86</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>507</v>
+      </c>
+      <c r="AC6" t="n">
         <v>1637.56</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AD6" t="n">
         <v>414</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AE6" t="n">
         <v>1550.15</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AF6" t="n">
         <v>316</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AG6" t="n">
         <v>1350.19</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AH6" t="n">
         <v>268</v>
       </c>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="n">
+      <c r="AI6" t="n">
+        <v>1270.75</v>
+      </c>
+      <c r="AJ6" t="n">
         <v>829</v>
       </c>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="n">
+      <c r="AK6" t="n">
+        <v>5066.24</v>
+      </c>
+      <c r="AL6" t="n">
         <v>374</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="AM6" t="n">
         <v>3226.85</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="AN6" t="n">
         <v>176</v>
       </c>
-      <c r="AM6" t="n">
+      <c r="AO6" t="n">
         <v>1954</v>
       </c>
-      <c r="AN6" t="n">
-        <v>16</v>
-      </c>
-      <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="n">
-        <v>13</v>
+        <v>76</v>
       </c>
       <c r="AQ6" t="n">
+        <v>1040.41</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>73</v>
+      </c>
+      <c r="AS6" t="n">
         <v>1258.63</v>
       </c>
-      <c r="AR6" t="n">
+      <c r="AT6" t="n">
         <v>29</v>
       </c>
-      <c r="AS6" t="n">
+      <c r="AU6" t="n">
         <v>649.49</v>
       </c>
-      <c r="AT6" t="n">
+      <c r="AV6" t="n">
         <v>18</v>
       </c>
-      <c r="AU6" t="n">
+      <c r="AW6" t="n">
         <v>491.28</v>
       </c>
-      <c r="AV6" t="n">
+      <c r="AX6" t="n">
         <v>17</v>
       </c>
-      <c r="AW6" t="n">
+      <c r="AY6" t="n">
         <v>599.09</v>
       </c>
-      <c r="AX6" t="n">
+      <c r="AZ6" t="n">
         <v>6</v>
       </c>
-      <c r="AY6" t="n">
+      <c r="BA6" t="n">
         <v>271.13</v>
       </c>
-      <c r="AZ6" t="n">
+      <c r="BB6" t="n">
         <v>11</v>
       </c>
-      <c r="BA6" t="n">
+      <c r="BC6" t="n">
         <v>736.87</v>
-      </c>
-      <c r="BB6" t="n">
-        <v>2</v>
-      </c>
-      <c r="BC6" t="n">
-        <v>168.25</v>
       </c>
       <c r="BD6" t="n">
         <v>2</v>
       </c>
-      <c r="BE6" t="inlineStr"/>
+      <c r="BE6" t="n">
+        <v>168.25</v>
+      </c>
       <c r="BF6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG6" t="n">
+        <v>273.19</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI6" t="n">
         <v>186.79</v>
       </c>
-      <c r="BH6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI6" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ6" t="n">
         <v>0</v>
       </c>
       <c r="BK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM6" t="n">
         <v>1351.57</v>
       </c>
-      <c r="BL6" t="n">
+      <c r="BN6" t="n">
         <v>2</v>
       </c>
-      <c r="BM6" t="inlineStr"/>
-      <c r="BN6" t="n">
-        <v>0</v>
-      </c>
       <c r="BO6" t="n">
-        <v>23.02</v>
+        <v>1447.99</v>
       </c>
       <c r="BP6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BQ6" t="n">
-        <v>0</v>
+        <v>1023.02</v>
       </c>
       <c r="BR6" t="n">
         <v>0</v>
@@ -1956,7 +1980,7 @@
         <v>14539</v>
       </c>
       <c r="BU6" t="n">
-        <v>0</v>
+        <v>35935.25</v>
       </c>
       <c r="BV6" t="inlineStr">
         <is>
@@ -2003,7 +2027,9 @@
       <c r="H7" t="n">
         <v>213</v>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>35.34</v>
+      </c>
       <c r="J7" t="n">
         <v>160</v>
       </c>
@@ -2062,99 +2088,103 @@
         <v>246</v>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>794.73</v>
       </c>
       <c r="AD7" t="n">
         <v>244</v>
       </c>
       <c r="AE7" t="n">
-        <v>0</v>
+        <v>924.3</v>
       </c>
       <c r="AF7" t="n">
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="AG7" t="n">
-        <v>0</v>
+        <v>691.55</v>
       </c>
       <c r="AH7" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="AI7" t="n">
-        <v>0</v>
+        <v>954.59</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0</v>
+        <v>636</v>
       </c>
       <c r="AK7" t="n">
-        <v>0</v>
+        <v>3897.32</v>
       </c>
       <c r="AL7" t="n">
-        <v>0</v>
+        <v>256</v>
       </c>
       <c r="AM7" t="n">
-        <v>0</v>
+        <v>2187.12</v>
       </c>
       <c r="AN7" t="n">
+        <v>102</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>1147.61</v>
+      </c>
+      <c r="AP7" t="n">
         <v>66</v>
       </c>
-      <c r="AO7" t="n">
+      <c r="AQ7" t="n">
         <v>893.71</v>
       </c>
-      <c r="AP7" t="n">
+      <c r="AR7" t="n">
         <v>40</v>
       </c>
-      <c r="AQ7" t="n">
+      <c r="AS7" t="n">
         <v>698.91</v>
       </c>
-      <c r="AR7" t="n">
+      <c r="AT7" t="n">
         <v>14</v>
       </c>
-      <c r="AS7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT7" t="n">
+      <c r="AU7" t="n">
+        <v>317.92</v>
+      </c>
+      <c r="AV7" t="n">
         <v>3</v>
       </c>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="n">
+      <c r="AW7" t="n">
+        <v>82.47</v>
+      </c>
+      <c r="AX7" t="n">
         <v>5</v>
       </c>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="n">
+      <c r="AY7" t="n">
+        <v>159.5</v>
+      </c>
+      <c r="AZ7" t="n">
         <v>3</v>
       </c>
-      <c r="AY7" t="n">
+      <c r="BA7" t="n">
         <v>128.61</v>
       </c>
-      <c r="AZ7" t="n">
+      <c r="BB7" t="n">
         <v>5</v>
       </c>
-      <c r="BA7" t="n">
+      <c r="BC7" t="n">
         <v>328.41</v>
       </c>
-      <c r="BB7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC7" t="n">
+      <c r="BD7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE7" t="n">
         <v>84</v>
       </c>
-      <c r="BD7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE7" t="n">
+      <c r="BF7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG7" t="n">
         <v>384.51</v>
       </c>
-      <c r="BF7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG7" t="n">
+      <c r="BH7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI7" t="n">
         <v>161.48</v>
-      </c>
-      <c r="BH7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI7" t="n">
-        <v>0</v>
       </c>
       <c r="BJ7" t="n">
         <v>0</v>
@@ -2189,7 +2219,9 @@
       <c r="BT7" t="n">
         <v>4988</v>
       </c>
-      <c r="BU7" t="inlineStr"/>
+      <c r="BU7" t="n">
+        <v>17496.23</v>
+      </c>
       <c r="BV7" t="inlineStr">
         <is>
           <t>C</t>
@@ -2245,7 +2277,7 @@
         <v>57.7</v>
       </c>
       <c r="L8" t="n">
-        <v>13</v>
+        <v>193</v>
       </c>
       <c r="M8" t="n">
         <v>69.56999999999999</v>
@@ -2329,82 +2361,82 @@
         <v>664.55</v>
       </c>
       <c r="AN8" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="AO8" t="n">
-        <v>0</v>
+        <v>627.37</v>
       </c>
       <c r="AP8" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="AQ8" t="n">
+        <v>450.27</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>40</v>
+      </c>
+      <c r="AS8" t="n">
         <v>695.63</v>
       </c>
-      <c r="AR8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>0</v>
-      </c>
       <c r="AT8" t="n">
+        <v>26</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>585.26</v>
+      </c>
+      <c r="AV8" t="n">
         <v>19</v>
       </c>
-      <c r="AU8" t="n">
+      <c r="AW8" t="n">
         <v>527.02</v>
       </c>
-      <c r="AV8" t="n">
+      <c r="AX8" t="n">
         <v>15</v>
       </c>
-      <c r="AW8" t="n">
+      <c r="AY8" t="n">
         <v>509.01</v>
       </c>
-      <c r="AX8" t="n">
+      <c r="AZ8" t="n">
         <v>4</v>
       </c>
-      <c r="AY8" t="n">
+      <c r="BA8" t="n">
         <v>184.57</v>
       </c>
-      <c r="AZ8" t="n">
+      <c r="BB8" t="n">
         <v>7</v>
       </c>
-      <c r="BA8" t="n">
+      <c r="BC8" t="n">
         <v>422.07</v>
-      </c>
-      <c r="BB8" t="n">
-        <v>4</v>
-      </c>
-      <c r="BC8" t="n">
-        <v>332.19</v>
       </c>
       <c r="BD8" t="n">
         <v>4</v>
       </c>
       <c r="BE8" t="n">
+        <v>332.19</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BG8" t="n">
         <v>536.48</v>
       </c>
-      <c r="BF8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG8" t="n">
+      <c r="BH8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI8" t="n">
         <v>157.57</v>
       </c>
-      <c r="BH8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI8" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL8" t="n">
         <v>2</v>
       </c>
-      <c r="BK8" t="n">
+      <c r="BM8" t="n">
         <v>760.97</v>
-      </c>
-      <c r="BL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM8" t="n">
-        <v>0</v>
       </c>
       <c r="BN8" t="n">
         <v>0</v>
@@ -2428,7 +2460,7 @@
         <v>2864</v>
       </c>
       <c r="BU8" t="n">
-        <v>703.9</v>
+        <v>9703.9</v>
       </c>
       <c r="BV8" t="inlineStr">
         <is>
@@ -2461,7 +2493,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -2527,122 +2559,124 @@
         <v>287.67</v>
       </c>
       <c r="Z9" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="AA9" t="n">
-        <v>0</v>
+        <v>219.51</v>
       </c>
       <c r="AB9" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="AC9" t="n">
-        <v>0</v>
+        <v>257.38</v>
       </c>
       <c r="AD9" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="AE9" t="n">
-        <v>0</v>
+        <v>252.69</v>
       </c>
       <c r="AF9" t="n">
+        <v>46</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>196.54</v>
+      </c>
+      <c r="AH9" t="n">
         <v>44</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="AI9" t="n">
         <v>209.81</v>
       </c>
-      <c r="AH9" t="n">
+      <c r="AJ9" t="n">
         <v>182</v>
       </c>
-      <c r="AI9" t="n">
+      <c r="AK9" t="n">
         <v>1142.3</v>
       </c>
-      <c r="AJ9" t="n">
+      <c r="AL9" t="n">
         <v>170</v>
       </c>
-      <c r="AK9" t="n">
+      <c r="AM9" t="n">
         <v>1476.08</v>
       </c>
-      <c r="AL9" t="n">
+      <c r="AN9" t="n">
         <v>108</v>
       </c>
-      <c r="AM9" t="n">
+      <c r="AO9" t="n">
         <v>1214.81</v>
       </c>
-      <c r="AN9" t="n">
+      <c r="AP9" t="n">
         <v>76</v>
       </c>
-      <c r="AO9" t="n">
+      <c r="AQ9" t="n">
         <v>1045.6</v>
       </c>
-      <c r="AP9" t="n">
+      <c r="AR9" t="n">
         <v>114</v>
       </c>
-      <c r="AQ9" t="n">
+      <c r="AS9" t="n">
         <v>1937.56</v>
       </c>
-      <c r="AR9" t="n">
+      <c r="AT9" t="n">
         <v>67</v>
       </c>
-      <c r="AS9" t="n">
+      <c r="AU9" t="n">
         <v>1518.43</v>
       </c>
-      <c r="AT9" t="n">
+      <c r="AV9" t="n">
         <v>32</v>
       </c>
-      <c r="AU9" t="n">
+      <c r="AW9" t="n">
         <v>863.98</v>
       </c>
-      <c r="AV9" t="n">
+      <c r="AX9" t="n">
         <v>53</v>
       </c>
-      <c r="AW9" t="n">
+      <c r="AY9" t="n">
         <v>1826.74</v>
       </c>
-      <c r="AX9" t="n">
+      <c r="AZ9" t="n">
         <v>32</v>
       </c>
-      <c r="AY9" t="inlineStr"/>
-      <c r="AZ9" t="n">
+      <c r="BA9" t="n">
+        <v>1433.39</v>
+      </c>
+      <c r="BB9" t="n">
         <v>36</v>
       </c>
-      <c r="BA9" t="n">
+      <c r="BC9" t="n">
         <v>2164.63</v>
       </c>
-      <c r="BB9" t="n">
+      <c r="BD9" t="n">
         <v>22</v>
       </c>
-      <c r="BC9" t="n">
+      <c r="BE9" t="n">
         <v>1919.63</v>
       </c>
-      <c r="BD9" t="n">
+      <c r="BF9" t="n">
         <v>20</v>
       </c>
-      <c r="BE9" t="n">
+      <c r="BG9" t="n">
         <v>2532.72</v>
       </c>
-      <c r="BF9" t="n">
+      <c r="BH9" t="n">
         <v>6</v>
       </c>
-      <c r="BG9" t="n">
+      <c r="BI9" t="n">
         <v>1015.95</v>
       </c>
-      <c r="BH9" t="n">
+      <c r="BJ9" t="n">
         <v>3</v>
       </c>
-      <c r="BI9" t="n">
+      <c r="BK9" t="n">
         <v>668.21</v>
       </c>
-      <c r="BJ9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK9" t="n">
+      <c r="BL9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM9" t="n">
         <v>886.59</v>
-      </c>
-      <c r="BL9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM9" t="n">
-        <v>0</v>
       </c>
       <c r="BN9" t="n">
         <v>0</v>
@@ -2705,12 +2739,14 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="G10" t="n">
         <v>5.85</v>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>236</v>
+      </c>
       <c r="I10" t="n">
         <v>40.3</v>
       </c>
@@ -2775,107 +2811,119 @@
         <v>560.21</v>
       </c>
       <c r="AD10" t="n">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="AE10" t="n">
-        <v>0</v>
+        <v>532.76</v>
       </c>
       <c r="AF10" t="n">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="AG10" t="n">
-        <v>0</v>
+        <v>517.63</v>
       </c>
       <c r="AH10" t="n">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="AI10" t="n">
-        <v>0</v>
+        <v>746.54</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0</v>
+        <v>538</v>
       </c>
       <c r="AK10" t="n">
-        <v>0</v>
+        <v>3340.83</v>
       </c>
       <c r="AL10" t="n">
+        <v>396</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>3394.38</v>
+      </c>
+      <c r="AN10" t="n">
         <v>166</v>
       </c>
-      <c r="AM10" t="inlineStr"/>
-      <c r="AN10" t="n">
+      <c r="AO10" t="n">
+        <v>1853.82</v>
+      </c>
+      <c r="AP10" t="n">
         <v>111</v>
       </c>
-      <c r="AO10" t="n">
+      <c r="AQ10" t="n">
         <v>1509.31</v>
       </c>
-      <c r="AP10" t="n">
+      <c r="AR10" t="n">
         <v>110</v>
       </c>
-      <c r="AQ10" t="n">
+      <c r="AS10" t="n">
         <v>1854.09</v>
       </c>
-      <c r="AR10" t="n">
+      <c r="AT10" t="n">
         <v>57</v>
       </c>
-      <c r="AS10" t="n">
+      <c r="AU10" t="n">
         <v>1269.5</v>
       </c>
-      <c r="AT10" t="n">
+      <c r="AV10" t="n">
         <v>34</v>
       </c>
-      <c r="AU10" t="n">
+      <c r="AW10" t="n">
         <v>921.42</v>
       </c>
-      <c r="AV10" t="n">
+      <c r="AX10" t="n">
         <v>45</v>
       </c>
-      <c r="AW10" t="inlineStr"/>
-      <c r="AX10" t="n">
+      <c r="AY10" t="n">
+        <v>1542.62</v>
+      </c>
+      <c r="AZ10" t="n">
         <v>27</v>
       </c>
-      <c r="AY10" t="n">
+      <c r="BA10" t="n">
         <v>1184.81</v>
       </c>
-      <c r="AZ10" t="inlineStr"/>
-      <c r="BA10" t="n">
+      <c r="BB10" t="n">
+        <v>27</v>
+      </c>
+      <c r="BC10" t="n">
         <v>1644.9</v>
       </c>
-      <c r="BB10" t="n">
+      <c r="BD10" t="n">
         <v>29</v>
       </c>
-      <c r="BC10" t="inlineStr"/>
-      <c r="BD10" t="n">
+      <c r="BE10" t="n">
+        <v>2456.66</v>
+      </c>
+      <c r="BF10" t="n">
         <v>22</v>
       </c>
-      <c r="BE10" t="n">
+      <c r="BG10" t="n">
         <v>2673.82</v>
       </c>
-      <c r="BF10" t="n">
+      <c r="BH10" t="n">
         <v>9</v>
       </c>
-      <c r="BG10" t="n">
+      <c r="BI10" t="n">
         <v>1477.75</v>
       </c>
-      <c r="BH10" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI10" t="n">
+      <c r="BJ10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK10" t="n">
         <v>239.88</v>
       </c>
-      <c r="BJ10" t="inlineStr"/>
-      <c r="BK10" t="inlineStr"/>
       <c r="BL10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>1066.93</v>
+      </c>
+      <c r="BN10" t="n">
         <v>1</v>
       </c>
-      <c r="BM10" t="n">
+      <c r="BO10" t="n">
         <v>560.65</v>
       </c>
-      <c r="BN10" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO10" t="n">
-        <v>0</v>
-      </c>
       <c r="BP10" t="n">
         <v>0</v>
       </c>
@@ -2888,7 +2936,9 @@
       <c r="BS10" t="n">
         <v>0</v>
       </c>
-      <c r="BT10" t="inlineStr"/>
+      <c r="BT10" t="n">
+        <v>5206</v>
+      </c>
       <c r="BU10" t="n">
         <v>32566.84</v>
       </c>
@@ -2973,7 +3023,9 @@
       <c r="T11" t="n">
         <v>610</v>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="n">
+        <v>757.89</v>
+      </c>
       <c r="V11" t="n">
         <v>475</v>
       </c>
@@ -2989,7 +3041,9 @@
       <c r="Z11" t="n">
         <v>217</v>
       </c>
-      <c r="AA11" t="inlineStr"/>
+      <c r="AA11" t="n">
+        <v>589.76</v>
+      </c>
       <c r="AB11" t="n">
         <v>145</v>
       </c>
@@ -3015,7 +3069,7 @@
         <v>506.24</v>
       </c>
       <c r="AJ11" t="n">
-        <v>317</v>
+        <v>377</v>
       </c>
       <c r="AK11" t="n">
         <v>2328.83</v>
@@ -3030,83 +3084,85 @@
         <v>194</v>
       </c>
       <c r="AO11" t="n">
-        <v>0</v>
+        <v>2165.49</v>
       </c>
       <c r="AP11" t="n">
-        <v>0</v>
+        <v>134</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0</v>
+        <v>1843.39</v>
       </c>
       <c r="AR11" t="n">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="AS11" t="n">
-        <v>0</v>
+        <v>3114.09</v>
       </c>
       <c r="AT11" t="n">
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="AU11" t="n">
+        <v>2484.34</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>63</v>
+      </c>
+      <c r="AW11" t="n">
         <v>1731.08</v>
       </c>
-      <c r="AV11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW11" t="n">
+      <c r="AX11" t="n">
+        <v>84</v>
+      </c>
+      <c r="AY11" t="n">
         <v>2913.53</v>
       </c>
-      <c r="AX11" t="n">
+      <c r="AZ11" t="n">
         <v>77</v>
       </c>
-      <c r="AY11" t="inlineStr"/>
-      <c r="AZ11" t="n">
+      <c r="BA11" t="n">
+        <v>3435.09</v>
+      </c>
+      <c r="BB11" t="n">
         <v>87</v>
       </c>
-      <c r="BA11" t="n">
+      <c r="BC11" t="n">
         <v>5222.46</v>
       </c>
-      <c r="BB11" t="n">
+      <c r="BD11" t="n">
         <v>42</v>
       </c>
-      <c r="BC11" t="n">
+      <c r="BE11" t="n">
         <v>3614.44</v>
       </c>
-      <c r="BD11" t="n">
+      <c r="BF11" t="n">
         <v>39</v>
       </c>
-      <c r="BE11" t="n">
+      <c r="BG11" t="n">
         <v>4751.93</v>
       </c>
-      <c r="BF11" t="n">
+      <c r="BH11" t="n">
         <v>14</v>
       </c>
-      <c r="BG11" t="n">
+      <c r="BI11" t="n">
         <v>2495.5</v>
       </c>
-      <c r="BH11" t="n">
+      <c r="BJ11" t="n">
         <v>4</v>
       </c>
-      <c r="BI11" t="n">
+      <c r="BK11" t="n">
         <v>890.9400000000001</v>
       </c>
-      <c r="BJ11" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK11" t="n">
+      <c r="BL11" t="n">
+        <v>5</v>
+      </c>
+      <c r="BM11" t="n">
         <v>1604.44</v>
       </c>
-      <c r="BL11" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM11" t="n">
+      <c r="BN11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO11" t="n">
         <v>1267.35</v>
-      </c>
-      <c r="BN11" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO11" t="n">
-        <v>0</v>
       </c>
       <c r="BP11" t="n">
         <v>0</v>
@@ -3123,7 +3179,9 @@
       <c r="BT11" t="n">
         <v>5618</v>
       </c>
-      <c r="BU11" t="inlineStr"/>
+      <c r="BU11" t="n">
+        <v>48060.42</v>
+      </c>
       <c r="BV11" t="inlineStr">
         <is>
           <t>P</t>

</xml_diff>